<commit_message>
doubled all damage/prevent, buffed thunderbolt, fixed image names
</commit_message>
<xml_diff>
--- a/acolyte_cards.xlsx
+++ b/acolyte_cards.xlsx
@@ -33,7 +33,7 @@
     <t xml:space="preserve">Holy Light</t>
   </si>
   <si>
-    <t xml:space="preserve">Heal 1. If healing another player: gain 1 resource.</t>
+    <t xml:space="preserve">Heal 2. If healing another player: gain 1 resource.</t>
   </si>
   <si>
     <t>cardimages/restore.png</t>
@@ -51,7 +51,7 @@
     <t>Consecration</t>
   </si>
   <si>
-    <t xml:space="preserve">Deal 1 to everyone; repeat next turn.</t>
+    <t xml:space="preserve">Deal 2 to everyone; repeat next turn.</t>
   </si>
   <si>
     <t>cardimages/seal_of_wisdom.png</t>
@@ -78,7 +78,7 @@
     <t xml:space="preserve">Righteous Defense</t>
   </si>
   <si>
-    <t xml:space="preserve">Prevent 3. Take all damage players would take. Gather 1 per damage taken.</t>
+    <t xml:space="preserve">Prevent 6. Take all damage players would take. Gather 1 per damage taken.</t>
   </si>
   <si>
     <t>cardimages/judgement.png</t>
@@ -96,7 +96,7 @@
     <t xml:space="preserve">Execution Sentence</t>
   </si>
   <si>
-    <t xml:space="preserve">In 3 turns, deal 5 damage to monster.</t>
+    <t xml:space="preserve">In 3 turns, deal 10 damage to monster.</t>
   </si>
   <si>
     <t>cardimages/sacred_shield.png</t>
@@ -105,7 +105,7 @@
     <t xml:space="preserve">Sacred Shield</t>
   </si>
   <si>
-    <t xml:space="preserve">Prevent 2 this turn and 2 next turn.</t>
+    <t xml:space="preserve">Prevent 4 this turn and 4 next turn.</t>
   </si>
   <si>
     <t>cardimages/faceup_synergy.png</t>
@@ -651,6 +651,7 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="29.28125"/>
+    <col bestFit="1" min="2" max="2" width="17.28125"/>
     <col customWidth="1" min="3" max="3" width="108.421875"/>
   </cols>
   <sheetData>

</xml_diff>